<commit_message>
Write a backup only when the data changed
Each workbook embeds the time it was taken, so rewriting an unchanged one
produced a fresh file every night. That meant a commit a day regardless of
whether anything happened, burying the real versions. On an unchanged day
nothing is written now; the existing latest.xlsx is still accurate, and the
Actions log is the record that the backup ran.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backups/latest.xlsx
+++ b/backups/latest.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Monday" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tuesday" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Wednesday" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Thursday" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Friday" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Checkouts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Changes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Rooms" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="About" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monday" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tuesday" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wednesday" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thursday" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Friday" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkouts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20191,7 +20191,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-15 21:32 UTC</t>
+          <t>2026-09-15 21:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>